<commit_message>
Nueva Rama y readme Actualizado
</commit_message>
<xml_diff>
--- a/registros_dorsales.xlsx
+++ b/registros_dorsales.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,14 +449,27 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
+      <c r="B2" t="n">
+        <v>100</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2025-10-29 17:14:03</t>
+          <t>2025-10-30 16:48:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>205</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2025-10-30 16:49:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Se termino la nueva interfaz y se agrego el atributo de categoria al registro de los dorsales al igual que en la interfaz
</commit_message>
<xml_diff>
--- a/registros_dorsales.xlsx
+++ b/registros_dorsales.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,10 +451,15 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Categoría</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>HoraLlegada</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
@@ -476,15 +481,20 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Ramods</t>
+          <t>Ramos</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>00:00:08</t>
+          <t>MASTER A</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
+        <is>
+          <t>00:00:09</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>Registrado</t>
         </is>

</xml_diff>

<commit_message>
Servidor implementado por categoria y generos
</commit_message>
<xml_diff>
--- a/registros_dorsales.xlsx
+++ b/registros_dorsales.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,20 +451,25 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Género</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Categoría</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Distancia</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>HoraLlegada</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
@@ -475,34 +480,39 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>205</v>
+        <v>101</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Karen Andrea </t>
+          <t xml:space="preserve">Marlon Adrian </t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Araujo</t>
+          <t>Casco Manobanda</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>MASTER A</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>10K</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>00:00:03</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Registrado</t>
         </is>
@@ -513,34 +523,39 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>134</v>
+        <v>330</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Jeremy Ariel</t>
+          <t xml:space="preserve">Fernando Santiago </t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cando Tapia </t>
+          <t>Villalba Salazar</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>JUVENIL</t>
+          <t>FEMENINO</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>10K</t>
+          <t>MASTER A</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>00:00:09</t>
+          <t>20K</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
+        <is>
+          <t>00:00:06</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>Registrado</t>
         </is>
@@ -551,36 +566,21 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>101</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Marlon Adrian </t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Casco Manobanda</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>MASTER A</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>10K</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>00:00:13</t>
-        </is>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Registrado</t>
+          <t>00:00:10</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>No encontrado</t>
         </is>
       </c>
     </row>
@@ -589,34 +589,39 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>330</v>
+        <v>205</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fernando Santiago </t>
+          <t xml:space="preserve">Karen Andrea </t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Villalba Salazar</t>
+          <t>Araujo</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>FEMENINO</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>MASTER A</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>20K</t>
-        </is>
-      </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>00:00:16</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
+        <is>
+          <t>00:00:27</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>Registrado</t>
         </is>
@@ -641,20 +646,25 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>INFANTIL A</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>2K</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>00:00:20</t>
-        </is>
-      </c>
       <c r="H6" t="inlineStr">
+        <is>
+          <t>00:00:34</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>Registrado</t>
         </is>
@@ -664,23 +674,110 @@
       <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
+      <c r="B7" t="n">
+        <v>220</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delia Fanny </t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Mullo Gualan</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>FEMENINO</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>MASTER B</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>00:00:23</t>
+          <t>10K</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
+          <t>00:00:34</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Registrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>95</v>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>00:00:46</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
           <t>No encontrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>023</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Amyra </t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Aguagallo Parra</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>FEMENINO</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>INFANTIL A</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2K</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>00:01:27</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Registrado</t>
         </is>
       </c>
     </row>

</xml_diff>